<commit_message>
Fix #NAME? formula parsing issue and restore clean HTML5 design
</commit_message>
<xml_diff>
--- a/Assignment 3 - Text , Logical, Date, Sumifs etc...xlsx
+++ b/Assignment 3 - Text , Logical, Date, Sumifs etc...xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucky\Desktop\Advance Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95AC37F8-5294-47BF-8901-DF38A79ED50F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D35B3308-D450-4819-9A2A-776E0FEA851D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6474,14 +6474,14 @@
       </c>
       <c r="C3" s="40">
         <f ca="1">TODAY()</f>
-        <v>46241</v>
+        <v>46245</v>
       </c>
       <c r="F3" s="9" t="s">
         <v>70</v>
       </c>
       <c r="G3" s="40">
         <f ca="1">TODAY()-14</f>
-        <v>46227</v>
+        <v>46231</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
@@ -6490,14 +6490,14 @@
       </c>
       <c r="C4" s="41">
         <f ca="1">NOW()</f>
-        <v>46241.623535995372</v>
+        <v>46245.642577662038</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>72</v>
       </c>
       <c r="G4" s="41">
         <f ca="1">NOW()-14</f>
-        <v>46227.623535995372</v>
+        <v>46231.642577662038</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
@@ -6555,7 +6555,7 @@
       </c>
       <c r="I7" s="43" t="str">
         <f ca="1">DATEDIF(C7,$C$3,"Y")&amp;" Years, "&amp;DATEDIF(C7,$C$3,"YM")&amp;" Months, "&amp;DATEDIF(C7,$C$3,"MD")&amp;" Days"</f>
-        <v>26 Years, 8 Months, 24 Days</v>
+        <v>26 Years, 8 Months, 28 Days</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
@@ -6587,7 +6587,7 @@
       </c>
       <c r="I8" s="43" t="str">
         <f t="shared" ref="I8:I18" ca="1" si="5">DATEDIF(C8,$C$3,"Y")&amp;" Years, "&amp;DATEDIF(C8,$C$3,"YM")&amp;" Months, "&amp;DATEDIF(C8,$C$3,"MD")&amp;" Days"</f>
-        <v>25 Years, 2 Months, 22 Days</v>
+        <v>25 Years, 2 Months, 26 Days</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
@@ -6619,7 +6619,7 @@
       </c>
       <c r="I9" s="43" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>22 Years, 8 Months, 17 Days</v>
+        <v>22 Years, 8 Months, 21 Days</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
@@ -6651,7 +6651,7 @@
       </c>
       <c r="I10" s="43" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>22 Years, 3 Months, 1 Days</v>
+        <v>22 Years, 3 Months, 5 Days</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
@@ -6683,7 +6683,7 @@
       </c>
       <c r="I11" s="43" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>21 Years, 4 Months, 0 Days</v>
+        <v>21 Years, 4 Months, 4 Days</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
@@ -6715,7 +6715,7 @@
       </c>
       <c r="I12" s="43" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>17 Years, 6 Months, 5 Days</v>
+        <v>17 Years, 6 Months, 9 Days</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="I13" s="43" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>16 Years, 2 Months, 6 Days</v>
+        <v>16 Years, 2 Months, 10 Days</v>
       </c>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
@@ -6779,7 +6779,7 @@
       </c>
       <c r="I14" s="43" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>15 Years, 8 Months, 25 Days</v>
+        <v>15 Years, 8 Months, 29 Days</v>
       </c>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.25">
@@ -6811,7 +6811,7 @@
       </c>
       <c r="I15" s="43" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>15 Years, 6 Months, 7 Days</v>
+        <v>15 Years, 6 Months, 11 Days</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
@@ -6843,7 +6843,7 @@
       </c>
       <c r="I16" s="43" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>13 Years, 3 Months, 1 Days</v>
+        <v>13 Years, 3 Months, 5 Days</v>
       </c>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
@@ -6875,7 +6875,7 @@
       </c>
       <c r="I17" s="43" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>11 Years, 6 Months, 15 Days</v>
+        <v>11 Years, 6 Months, 19 Days</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.25">
@@ -6907,7 +6907,7 @@
       </c>
       <c r="I18" s="43" t="str">
         <f t="shared" ca="1" si="5"/>
-        <v>11 Years, 3 Months, 8 Days</v>
+        <v>11 Years, 3 Months, 12 Days</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">

</xml_diff>